<commit_message>
Add Catalog Demand list: provisioning script, runner wiring, and schema workbook
The out-of-catalog hand-off log was live and written by the RITM validation flow, but no provisioning script created it. Add 18-catalog-demand.ps1 matching the live schema, wire it into both provisioning runners, and document it as sheet 11 in the schema workbook.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sharepoint-itsm-schema.xlsx
+++ b/sharepoint-itsm-schema.xlsx
@@ -19,9 +19,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Knowledge Base" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Approvals" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Priority Matrix" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choices Reference" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Matrix Data" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance Notes" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Catalog Demand" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choices Reference" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Matrix Data" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance Notes" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -601,7 +602,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-29 (rev. 2026-06-08)</t>
         </is>
       </c>
     </row>
@@ -613,7 +614,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>10 SharePoint lists modelling the core of ServiceNow ITSM.</t>
+          <t>10 core ServiceNow lists + 1 operational list (Catalog Demand) = 11 documented here.</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2381,378 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>11. Catalog Demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Out-of-catalog demand log. One row per request the automation could not fulfil and handed off to the IT Service Desk queue. Written by the RITM-Validation-Triage flow (Create_CatalogDemand); triage DemandStatus to decide what to onboard into the catalog next. Operational list — not part of the core ServiceNow model in lists 1-10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Internal Name</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Display Name</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Column Type</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Default Value</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Choices / Lookup Target</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Indexed</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Purpose / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Demand Summary</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Auto-composed by Flow as "&lt;RITM#&gt; - &lt;resource&gt;".</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>RequestedItem</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Requested Item</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Catalog item name if one was matched, else the originating ticket title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>ResourceName</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Resource Name</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>The specific resource the requester named (license SKU, group, app), parsed from the request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>JobTypeGuess</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Job Type Guess</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Agent's best guess at the JobType this would map to if automated. Blank when it could not be inferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Requester</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Requester</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>UPN of the requester (text, from the RITM RequestedFor claim — not a Person column).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>RitmRef</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>RITM Ref</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Single line of text</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>RITM number the demand came from. Back-traces to the request and ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>DemandStatus</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Demand Status</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Choice</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>New; Reviewing; Onboarded; Declined</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Review state. New → Reviewing → Onboarded (added to catalog) or Declined.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>DemandNotes</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Demand Notes</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Multiple lines of text</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Agent's summary of what was wanted, plus reviewer notes. Plain text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Total columns: 8</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4216,6 +4588,78 @@
       </c>
       <c r="E125" s="7" t="inlineStr"/>
     </row>
+    <row r="126">
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>Catalog Demand</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>DemandStatus</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="n"/>
+      <c r="B127" s="9" t="n"/>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>Reviewing</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="n"/>
+      <c r="B128" s="9" t="n"/>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>Onboarded</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="9" t="n"/>
+      <c r="B129" s="9" t="n"/>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -4225,7 +4669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4549,7 +4993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4796,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4817,7 +5261,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10 SharePoint lists. List 9 (Approvals) and 10 (Priority Matrix) are optional.</t>
+          <t>11 SharePoint lists. Lists 1-10 model the core ServiceNow data model; list 11 (Catalog Demand) is an operational list written by the automation. List 9 (Approvals) and 10 (Priority Matrix) are optional.</t>
         </is>
       </c>
     </row>
@@ -5150,6 +5594,38 @@
       <c r="F14" s="9" t="inlineStr">
         <is>
           <t>9-row lookup. Skip if you hardcode the matrix in Flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>11. Catalog Demand</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>8 cols</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>→ Request Items (RitmRef, text)</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>LOW-MED (grows with unmet demand)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Operational. Out-of-catalog demand log written by RITM-Validation-Triage; triage to decide what to onboard.</t>
         </is>
       </c>
     </row>

</xml_diff>